<commit_message>
continue migration and sent water tank estimate for r to nabin sir
</commit_message>
<xml_diff>
--- a/2083_2084/estimate/budget maag estimate/Ward swasthya water tank/size water tank.xlsx
+++ b/2083_2084/estimate/budget maag estimate/Ward swasthya water tank/size water tank.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\2082_2083\2083_2084\estimate\budget maag estimate\Ward swasthya water tank\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C05AD076-0EDD-4CAD-8569-BFB0884326B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8CBBF8B-0EE1-4F07-B31B-BE9597E6C836}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10095" yWindow="0" windowWidth="10395" windowHeight="10905" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="WCR" sheetId="27" state="hidden" r:id="rId1"/>
@@ -3306,15 +3306,6 @@
     <xf numFmtId="0" fontId="64" fillId="0" borderId="19" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="43" fontId="64" fillId="0" borderId="19" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="48" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="64" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="50" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="50" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -3330,6 +3321,30 @@
     </xf>
     <xf numFmtId="0" fontId="50" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="43" fontId="64" fillId="0" borderId="19" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="64" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="63" fillId="32" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="63" fillId="32" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="63" fillId="32" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="58" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -3347,21 +3362,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="61" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="63" fillId="32" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="63" fillId="32" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="63" fillId="32" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="68" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -4626,60 +4626,60 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
-      <c r="A1" s="157" t="s">
+      <c r="A1" s="162" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="157"/>
-      <c r="C1" s="157"/>
-      <c r="D1" s="157"/>
-      <c r="E1" s="157"/>
-      <c r="F1" s="157"/>
-      <c r="G1" s="157"/>
-      <c r="H1" s="157"/>
-      <c r="I1" s="157"/>
-      <c r="J1" s="157"/>
+      <c r="B1" s="162"/>
+      <c r="C1" s="162"/>
+      <c r="D1" s="162"/>
+      <c r="E1" s="162"/>
+      <c r="F1" s="162"/>
+      <c r="G1" s="162"/>
+      <c r="H1" s="162"/>
+      <c r="I1" s="162"/>
+      <c r="J1" s="162"/>
     </row>
     <row r="2" spans="1:10" ht="25.5">
-      <c r="A2" s="158" t="s">
+      <c r="A2" s="163" t="s">
         <v>49</v>
       </c>
-      <c r="B2" s="158"/>
-      <c r="C2" s="158"/>
-      <c r="D2" s="158"/>
-      <c r="E2" s="158"/>
-      <c r="F2" s="158"/>
-      <c r="G2" s="158"/>
-      <c r="H2" s="158"/>
-      <c r="I2" s="158"/>
-      <c r="J2" s="158"/>
+      <c r="B2" s="163"/>
+      <c r="C2" s="163"/>
+      <c r="D2" s="163"/>
+      <c r="E2" s="163"/>
+      <c r="F2" s="163"/>
+      <c r="G2" s="163"/>
+      <c r="H2" s="163"/>
+      <c r="I2" s="163"/>
+      <c r="J2" s="163"/>
     </row>
     <row r="3" spans="1:10" ht="18.75">
-      <c r="A3" s="159" t="s">
+      <c r="A3" s="164" t="s">
         <v>50</v>
       </c>
-      <c r="B3" s="159"/>
-      <c r="C3" s="159"/>
-      <c r="D3" s="159"/>
-      <c r="E3" s="159"/>
-      <c r="F3" s="159"/>
-      <c r="G3" s="159"/>
-      <c r="H3" s="159"/>
-      <c r="I3" s="159"/>
-      <c r="J3" s="159"/>
+      <c r="B3" s="164"/>
+      <c r="C3" s="164"/>
+      <c r="D3" s="164"/>
+      <c r="E3" s="164"/>
+      <c r="F3" s="164"/>
+      <c r="G3" s="164"/>
+      <c r="H3" s="164"/>
+      <c r="I3" s="164"/>
+      <c r="J3" s="164"/>
     </row>
     <row r="4" spans="1:10">
-      <c r="A4" s="160" t="s">
+      <c r="A4" s="165" t="s">
         <v>51</v>
       </c>
-      <c r="B4" s="160"/>
-      <c r="C4" s="160"/>
-      <c r="D4" s="160"/>
-      <c r="E4" s="160"/>
-      <c r="F4" s="160"/>
-      <c r="G4" s="160"/>
-      <c r="H4" s="160"/>
-      <c r="I4" s="160"/>
-      <c r="J4" s="160"/>
+      <c r="B4" s="165"/>
+      <c r="C4" s="165"/>
+      <c r="D4" s="165"/>
+      <c r="E4" s="165"/>
+      <c r="F4" s="165"/>
+      <c r="G4" s="165"/>
+      <c r="H4" s="165"/>
+      <c r="I4" s="165"/>
+      <c r="J4" s="165"/>
     </row>
     <row r="5" spans="1:10">
       <c r="A5" s="12"/>
@@ -4698,33 +4698,33 @@
         <v>52</v>
       </c>
       <c r="B6" s="6"/>
-      <c r="C6" s="161" t="e">
+      <c r="C6" s="166" t="e">
         <f>E51</f>
         <v>#REF!</v>
       </c>
-      <c r="D6" s="162"/>
+      <c r="D6" s="167"/>
       <c r="E6" s="6"/>
       <c r="F6" s="6"/>
       <c r="G6" s="6" t="s">
         <v>53</v>
       </c>
       <c r="H6" s="6"/>
-      <c r="I6" s="161" t="e">
+      <c r="I6" s="166" t="e">
         <f>H51</f>
         <v>#REF!</v>
       </c>
-      <c r="J6" s="162"/>
+      <c r="J6" s="167"/>
     </row>
     <row r="7" spans="1:10">
       <c r="A7" s="7"/>
       <c r="B7" s="7"/>
-      <c r="C7" s="163"/>
-      <c r="D7" s="163"/>
-      <c r="E7" s="163"/>
-      <c r="F7" s="163"/>
-      <c r="H7" s="164"/>
-      <c r="I7" s="164"/>
-      <c r="J7" s="164"/>
+      <c r="C7" s="157"/>
+      <c r="D7" s="157"/>
+      <c r="E7" s="157"/>
+      <c r="F7" s="157"/>
+      <c r="H7" s="158"/>
+      <c r="I7" s="158"/>
+      <c r="J7" s="158"/>
     </row>
     <row r="8" spans="1:10" ht="16.5">
       <c r="A8" t="s">
@@ -4751,32 +4751,32 @@
       </c>
     </row>
     <row r="10" spans="1:10">
-      <c r="A10" s="165" t="s">
+      <c r="A10" s="159" t="s">
         <v>57</v>
       </c>
-      <c r="B10" s="165" t="s">
+      <c r="B10" s="159" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="167" t="s">
+      <c r="C10" s="161" t="s">
         <v>58</v>
       </c>
-      <c r="D10" s="167"/>
-      <c r="E10" s="167"/>
-      <c r="F10" s="167" t="s">
+      <c r="D10" s="161"/>
+      <c r="E10" s="161"/>
+      <c r="F10" s="161" t="s">
         <v>59</v>
       </c>
-      <c r="G10" s="167"/>
-      <c r="H10" s="167"/>
-      <c r="I10" s="165" t="s">
+      <c r="G10" s="161"/>
+      <c r="H10" s="161"/>
+      <c r="I10" s="159" t="s">
         <v>60</v>
       </c>
-      <c r="J10" s="165" t="s">
+      <c r="J10" s="159" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="11" spans="1:10">
-      <c r="A11" s="166"/>
-      <c r="B11" s="166"/>
+      <c r="A11" s="160"/>
+      <c r="B11" s="160"/>
       <c r="C11" s="14" t="s">
         <v>61</v>
       </c>
@@ -4795,8 +4795,8 @@
       <c r="H11" s="14" t="s">
         <v>63</v>
       </c>
-      <c r="I11" s="166"/>
-      <c r="J11" s="166"/>
+      <c r="I11" s="160"/>
+      <c r="J11" s="160"/>
     </row>
     <row r="12" spans="1:10" ht="15.75">
       <c r="A12" s="22">
@@ -5723,6 +5723,12 @@
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A3:J3"/>
+    <mergeCell ref="A4:J4"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="I6:J6"/>
     <mergeCell ref="C7:D7"/>
     <mergeCell ref="E7:F7"/>
     <mergeCell ref="H7:J7"/>
@@ -5732,12 +5738,6 @@
     <mergeCell ref="F10:H10"/>
     <mergeCell ref="I10:I11"/>
     <mergeCell ref="J10:J11"/>
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A2:J2"/>
-    <mergeCell ref="A3:J3"/>
-    <mergeCell ref="A4:J4"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="88" orientation="landscape" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
@@ -6016,94 +6016,94 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12">
-      <c r="A1" s="153" t="s">
+      <c r="A1" s="150" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="153"/>
-      <c r="C1" s="153"/>
-      <c r="D1" s="153"/>
-      <c r="E1" s="153"/>
-      <c r="F1" s="153"/>
-      <c r="G1" s="153"/>
-      <c r="H1" s="153"/>
-      <c r="I1" s="153"/>
-      <c r="J1" s="153"/>
-      <c r="K1" s="153"/>
+      <c r="B1" s="150"/>
+      <c r="C1" s="150"/>
+      <c r="D1" s="150"/>
+      <c r="E1" s="150"/>
+      <c r="F1" s="150"/>
+      <c r="G1" s="150"/>
+      <c r="H1" s="150"/>
+      <c r="I1" s="150"/>
+      <c r="J1" s="150"/>
+      <c r="K1" s="150"/>
       <c r="L1" s="109"/>
     </row>
     <row r="2" spans="1:12" ht="20.25">
-      <c r="A2" s="154" t="s">
+      <c r="A2" s="151" t="s">
         <v>16</v>
       </c>
-      <c r="B2" s="154"/>
-      <c r="C2" s="154"/>
-      <c r="D2" s="154"/>
-      <c r="E2" s="154"/>
-      <c r="F2" s="154"/>
-      <c r="G2" s="154"/>
-      <c r="H2" s="154"/>
-      <c r="I2" s="154"/>
-      <c r="J2" s="154"/>
-      <c r="K2" s="154"/>
+      <c r="B2" s="151"/>
+      <c r="C2" s="151"/>
+      <c r="D2" s="151"/>
+      <c r="E2" s="151"/>
+      <c r="F2" s="151"/>
+      <c r="G2" s="151"/>
+      <c r="H2" s="151"/>
+      <c r="I2" s="151"/>
+      <c r="J2" s="151"/>
+      <c r="K2" s="151"/>
       <c r="L2" s="118"/>
     </row>
     <row r="3" spans="1:12">
-      <c r="A3" s="153" t="s">
+      <c r="A3" s="150" t="s">
         <v>17</v>
       </c>
-      <c r="B3" s="153"/>
-      <c r="C3" s="153"/>
-      <c r="D3" s="153"/>
-      <c r="E3" s="153"/>
-      <c r="F3" s="153"/>
-      <c r="G3" s="153"/>
-      <c r="H3" s="153"/>
-      <c r="I3" s="153"/>
-      <c r="J3" s="153"/>
-      <c r="K3" s="153"/>
+      <c r="B3" s="150"/>
+      <c r="C3" s="150"/>
+      <c r="D3" s="150"/>
+      <c r="E3" s="150"/>
+      <c r="F3" s="150"/>
+      <c r="G3" s="150"/>
+      <c r="H3" s="150"/>
+      <c r="I3" s="150"/>
+      <c r="J3" s="150"/>
+      <c r="K3" s="150"/>
       <c r="L3" s="109"/>
     </row>
     <row r="4" spans="1:12">
-      <c r="A4" s="155" t="s">
+      <c r="A4" s="152" t="s">
         <v>22</v>
       </c>
-      <c r="B4" s="155"/>
-      <c r="C4" s="155"/>
-      <c r="D4" s="155"/>
-      <c r="E4" s="155"/>
-      <c r="F4" s="155"/>
-      <c r="G4" s="155"/>
-      <c r="H4" s="155"/>
-      <c r="I4" s="155"/>
-      <c r="J4" s="155"/>
-      <c r="K4" s="155"/>
+      <c r="B4" s="152"/>
+      <c r="C4" s="152"/>
+      <c r="D4" s="152"/>
+      <c r="E4" s="152"/>
+      <c r="F4" s="152"/>
+      <c r="G4" s="152"/>
+      <c r="H4" s="152"/>
+      <c r="I4" s="152"/>
+      <c r="J4" s="152"/>
+      <c r="K4" s="152"/>
     </row>
     <row r="5" spans="1:12" ht="20.25">
       <c r="A5" s="119" t="s">
         <v>139</v>
       </c>
       <c r="G5" s="4"/>
-      <c r="J5" s="156" t="s">
+      <c r="J5" s="153" t="s">
         <v>78</v>
       </c>
-      <c r="K5" s="156"/>
+      <c r="K5" s="153"/>
     </row>
     <row r="6" spans="1:12">
-      <c r="A6" s="151" t="s">
+      <c r="A6" s="148" t="s">
         <v>27</v>
       </c>
-      <c r="B6" s="151"/>
-      <c r="C6" s="151"/>
-      <c r="D6" s="151"/>
-      <c r="E6" s="151"/>
-      <c r="F6" s="151"/>
+      <c r="B6" s="148"/>
+      <c r="C6" s="148"/>
+      <c r="D6" s="148"/>
+      <c r="E6" s="148"/>
+      <c r="F6" s="148"/>
       <c r="G6" s="61"/>
-      <c r="H6" s="152" t="s">
+      <c r="H6" s="149" t="s">
         <v>140</v>
       </c>
-      <c r="I6" s="152"/>
-      <c r="J6" s="152"/>
-      <c r="K6" s="152"/>
+      <c r="I6" s="149"/>
+      <c r="J6" s="149"/>
+      <c r="K6" s="149"/>
     </row>
     <row r="7" spans="1:12">
       <c r="B7" s="3"/>
@@ -6679,7 +6679,7 @@
       <c r="J34" s="84"/>
       <c r="K34" s="81"/>
     </row>
-    <row r="35" spans="1:11" ht="30.75">
+    <row r="35" spans="1:11" ht="45.75">
       <c r="A35" s="77">
         <v>6</v>
       </c>
@@ -9452,10 +9452,10 @@
       <c r="B167" s="75" t="s">
         <v>12</v>
       </c>
-      <c r="C167" s="149" t="s">
+      <c r="C167" s="155" t="s">
         <v>66</v>
       </c>
-      <c r="D167" s="149"/>
+      <c r="D167" s="155"/>
       <c r="E167" s="75" t="s">
         <v>67</v>
       </c>
@@ -9471,11 +9471,11 @@
       <c r="B168" s="79" t="s">
         <v>13</v>
       </c>
-      <c r="C168" s="150">
+      <c r="C168" s="156">
         <f>+J165</f>
         <v>530004.91742540663</v>
       </c>
-      <c r="D168" s="150"/>
+      <c r="D168" s="156"/>
       <c r="E168" s="110"/>
       <c r="F168" s="108"/>
       <c r="G168" s="111"/>
@@ -9489,10 +9489,10 @@
       <c r="B169" s="79" t="s">
         <v>14</v>
       </c>
-      <c r="C169" s="150">
+      <c r="C169" s="156">
         <v>480000</v>
       </c>
-      <c r="D169" s="150"/>
+      <c r="D169" s="156"/>
       <c r="E169" s="112">
         <v>100</v>
       </c>
@@ -9508,11 +9508,11 @@
       <c r="B170" s="79" t="s">
         <v>19</v>
       </c>
-      <c r="C170" s="150">
+      <c r="C170" s="156">
         <f>0.95*C169</f>
         <v>456000</v>
       </c>
-      <c r="D170" s="150"/>
+      <c r="D170" s="156"/>
       <c r="E170" s="113">
         <f>C170/C168*100</f>
         <v>86.036937584485301</v>
@@ -9529,11 +9529,11 @@
       <c r="B171" s="79" t="s">
         <v>15</v>
       </c>
-      <c r="C171" s="150">
+      <c r="C171" s="156">
         <f>C168-C170</f>
         <v>74004.917425406631</v>
       </c>
-      <c r="D171" s="150"/>
+      <c r="D171" s="156"/>
       <c r="E171" s="113">
         <f>C171/C169*100</f>
         <v>15.417691130293049</v>
@@ -9550,11 +9550,11 @@
       <c r="B172" s="79" t="s">
         <v>20</v>
       </c>
-      <c r="C172" s="150">
+      <c r="C172" s="156">
         <f>E172*C169/100</f>
         <v>9600</v>
       </c>
-      <c r="D172" s="150"/>
+      <c r="D172" s="156"/>
       <c r="E172" s="113">
         <v>2</v>
       </c>
@@ -9570,11 +9570,11 @@
       <c r="B173" s="79" t="s">
         <v>21</v>
       </c>
-      <c r="C173" s="148">
+      <c r="C173" s="154">
         <f>E173*C169/100</f>
         <v>14400</v>
       </c>
-      <c r="D173" s="148"/>
+      <c r="D173" s="154"/>
       <c r="E173" s="113">
         <v>3</v>
       </c>
@@ -9590,6 +9590,13 @@
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="H6:K6"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A3:K3"/>
+    <mergeCell ref="A4:K4"/>
+    <mergeCell ref="J5:K5"/>
     <mergeCell ref="C173:D173"/>
     <mergeCell ref="C167:D167"/>
     <mergeCell ref="C168:D168"/>
@@ -9597,13 +9604,6 @@
     <mergeCell ref="C170:D170"/>
     <mergeCell ref="C171:D171"/>
     <mergeCell ref="C172:D172"/>
-    <mergeCell ref="A6:F6"/>
-    <mergeCell ref="H6:K6"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A3:K3"/>
-    <mergeCell ref="A4:K4"/>
-    <mergeCell ref="J5:K5"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.51181102362204722" right="0.51181102362204722" top="0.39370078740157483" bottom="0.70866141732283472" header="0.31496062992125984" footer="0.31496062992125984"/>
@@ -9802,94 +9802,94 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12">
-      <c r="A1" s="153" t="s">
+      <c r="A1" s="150" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="153"/>
-      <c r="C1" s="153"/>
-      <c r="D1" s="153"/>
-      <c r="E1" s="153"/>
-      <c r="F1" s="153"/>
-      <c r="G1" s="153"/>
-      <c r="H1" s="153"/>
-      <c r="I1" s="153"/>
-      <c r="J1" s="153"/>
-      <c r="K1" s="153"/>
+      <c r="B1" s="150"/>
+      <c r="C1" s="150"/>
+      <c r="D1" s="150"/>
+      <c r="E1" s="150"/>
+      <c r="F1" s="150"/>
+      <c r="G1" s="150"/>
+      <c r="H1" s="150"/>
+      <c r="I1" s="150"/>
+      <c r="J1" s="150"/>
+      <c r="K1" s="150"/>
       <c r="L1" s="109"/>
     </row>
     <row r="2" spans="1:12" ht="20.25">
-      <c r="A2" s="154" t="s">
+      <c r="A2" s="151" t="s">
         <v>16</v>
       </c>
-      <c r="B2" s="154"/>
-      <c r="C2" s="154"/>
-      <c r="D2" s="154"/>
-      <c r="E2" s="154"/>
-      <c r="F2" s="154"/>
-      <c r="G2" s="154"/>
-      <c r="H2" s="154"/>
-      <c r="I2" s="154"/>
-      <c r="J2" s="154"/>
-      <c r="K2" s="154"/>
+      <c r="B2" s="151"/>
+      <c r="C2" s="151"/>
+      <c r="D2" s="151"/>
+      <c r="E2" s="151"/>
+      <c r="F2" s="151"/>
+      <c r="G2" s="151"/>
+      <c r="H2" s="151"/>
+      <c r="I2" s="151"/>
+      <c r="J2" s="151"/>
+      <c r="K2" s="151"/>
       <c r="L2" s="118"/>
     </row>
     <row r="3" spans="1:12">
-      <c r="A3" s="153" t="s">
+      <c r="A3" s="150" t="s">
         <v>17</v>
       </c>
-      <c r="B3" s="153"/>
-      <c r="C3" s="153"/>
-      <c r="D3" s="153"/>
-      <c r="E3" s="153"/>
-      <c r="F3" s="153"/>
-      <c r="G3" s="153"/>
-      <c r="H3" s="153"/>
-      <c r="I3" s="153"/>
-      <c r="J3" s="153"/>
-      <c r="K3" s="153"/>
+      <c r="B3" s="150"/>
+      <c r="C3" s="150"/>
+      <c r="D3" s="150"/>
+      <c r="E3" s="150"/>
+      <c r="F3" s="150"/>
+      <c r="G3" s="150"/>
+      <c r="H3" s="150"/>
+      <c r="I3" s="150"/>
+      <c r="J3" s="150"/>
+      <c r="K3" s="150"/>
       <c r="L3" s="109"/>
     </row>
     <row r="4" spans="1:12">
-      <c r="A4" s="155" t="s">
+      <c r="A4" s="152" t="s">
         <v>22</v>
       </c>
-      <c r="B4" s="155"/>
-      <c r="C4" s="155"/>
-      <c r="D4" s="155"/>
-      <c r="E4" s="155"/>
-      <c r="F4" s="155"/>
-      <c r="G4" s="155"/>
-      <c r="H4" s="155"/>
-      <c r="I4" s="155"/>
-      <c r="J4" s="155"/>
-      <c r="K4" s="155"/>
+      <c r="B4" s="152"/>
+      <c r="C4" s="152"/>
+      <c r="D4" s="152"/>
+      <c r="E4" s="152"/>
+      <c r="F4" s="152"/>
+      <c r="G4" s="152"/>
+      <c r="H4" s="152"/>
+      <c r="I4" s="152"/>
+      <c r="J4" s="152"/>
+      <c r="K4" s="152"/>
     </row>
     <row r="5" spans="1:12" ht="20.25">
       <c r="A5" s="119" t="s">
         <v>139</v>
       </c>
       <c r="G5" s="4"/>
-      <c r="J5" s="156" t="s">
+      <c r="J5" s="153" t="s">
         <v>78</v>
       </c>
-      <c r="K5" s="156"/>
+      <c r="K5" s="153"/>
     </row>
     <row r="6" spans="1:12">
-      <c r="A6" s="151" t="s">
+      <c r="A6" s="148" t="s">
         <v>27</v>
       </c>
-      <c r="B6" s="151"/>
-      <c r="C6" s="151"/>
-      <c r="D6" s="151"/>
-      <c r="E6" s="151"/>
-      <c r="F6" s="151"/>
+      <c r="B6" s="148"/>
+      <c r="C6" s="148"/>
+      <c r="D6" s="148"/>
+      <c r="E6" s="148"/>
+      <c r="F6" s="148"/>
       <c r="G6" s="61"/>
-      <c r="H6" s="152" t="s">
+      <c r="H6" s="149" t="s">
         <v>140</v>
       </c>
-      <c r="I6" s="152"/>
-      <c r="J6" s="152"/>
-      <c r="K6" s="152"/>
+      <c r="I6" s="149"/>
+      <c r="J6" s="149"/>
+      <c r="K6" s="149"/>
     </row>
     <row r="7" spans="1:12">
       <c r="B7" s="3"/>
@@ -10620,7 +10620,7 @@
       <c r="J41" s="84"/>
       <c r="K41" s="81"/>
     </row>
-    <row r="42" spans="1:11" ht="30.75">
+    <row r="42" spans="1:11" ht="45.75">
       <c r="A42" s="77">
         <v>7</v>
       </c>
@@ -10661,10 +10661,7 @@
       </c>
       <c r="H43" s="80"/>
       <c r="I43" s="84"/>
-      <c r="J43" s="84">
-        <f>13.833/3.281</f>
-        <v>4.2160926546784516</v>
-      </c>
+      <c r="J43" s="84"/>
       <c r="K43" s="81"/>
     </row>
     <row r="44" spans="1:11">
@@ -12738,7 +12735,7 @@
       <c r="J137" s="80"/>
       <c r="K137" s="81"/>
     </row>
-    <row r="138" spans="1:11" ht="57">
+    <row r="138" spans="1:11" ht="69">
       <c r="A138" s="77">
         <v>16</v>
       </c>
@@ -16445,7 +16442,7 @@
       <c r="I312" s="84"/>
       <c r="J312" s="102">
         <f>SUM(J12:J311)</f>
-        <v>1198928.1474031552</v>
+        <v>1198923.9313105005</v>
       </c>
       <c r="K312" s="103"/>
     </row>
@@ -16467,10 +16464,10 @@
       <c r="B314" s="75" t="s">
         <v>12</v>
       </c>
-      <c r="C314" s="149" t="s">
+      <c r="C314" s="155" t="s">
         <v>66</v>
       </c>
-      <c r="D314" s="149"/>
+      <c r="D314" s="155"/>
       <c r="E314" s="75" t="s">
         <v>67</v>
       </c>
@@ -16486,11 +16483,11 @@
       <c r="B315" s="79" t="s">
         <v>13</v>
       </c>
-      <c r="C315" s="150">
+      <c r="C315" s="156">
         <f>+J312</f>
-        <v>1198928.1474031552</v>
-      </c>
-      <c r="D315" s="150"/>
+        <v>1198923.9313105005</v>
+      </c>
+      <c r="D315" s="156"/>
       <c r="E315" s="110"/>
       <c r="F315" s="108"/>
       <c r="G315" s="111"/>
@@ -16504,10 +16501,10 @@
       <c r="B316" s="79" t="s">
         <v>14</v>
       </c>
-      <c r="C316" s="150">
+      <c r="C316" s="156">
         <v>1050000</v>
       </c>
-      <c r="D316" s="150"/>
+      <c r="D316" s="156"/>
       <c r="E316" s="112">
         <v>100</v>
       </c>
@@ -16523,14 +16520,14 @@
       <c r="B317" s="79" t="s">
         <v>19</v>
       </c>
-      <c r="C317" s="150">
+      <c r="C317" s="156">
         <f>0.95*C316</f>
         <v>997500</v>
       </c>
-      <c r="D317" s="150"/>
+      <c r="D317" s="156"/>
       <c r="E317" s="113">
         <f>C317/C315*100</f>
-        <v>83.199314501086405</v>
+        <v>83.199607076795004</v>
       </c>
       <c r="F317" s="108"/>
       <c r="G317" s="111"/>
@@ -16544,14 +16541,14 @@
       <c r="B318" s="79" t="s">
         <v>15</v>
       </c>
-      <c r="C318" s="150">
+      <c r="C318" s="156">
         <f>C315-C317</f>
-        <v>201428.14740315522</v>
-      </c>
-      <c r="D318" s="150"/>
+        <v>201423.93131050048</v>
+      </c>
+      <c r="D318" s="156"/>
       <c r="E318" s="113">
         <f>C318/C316*100</f>
-        <v>19.183633086014783</v>
+        <v>19.183231553380999</v>
       </c>
       <c r="F318" s="108"/>
       <c r="G318" s="111"/>
@@ -16565,11 +16562,11 @@
       <c r="B319" s="79" t="s">
         <v>20</v>
       </c>
-      <c r="C319" s="150">
+      <c r="C319" s="156">
         <f>E319*C316/100</f>
         <v>21000</v>
       </c>
-      <c r="D319" s="150"/>
+      <c r="D319" s="156"/>
       <c r="E319" s="113">
         <v>2</v>
       </c>
@@ -16585,11 +16582,11 @@
       <c r="B320" s="79" t="s">
         <v>21</v>
       </c>
-      <c r="C320" s="148">
+      <c r="C320" s="154">
         <f>E320*C316/100</f>
         <v>31500</v>
       </c>
-      <c r="D320" s="148"/>
+      <c r="D320" s="154"/>
       <c r="E320" s="113">
         <v>3</v>
       </c>
@@ -16605,6 +16602,13 @@
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="C320:D320"/>
+    <mergeCell ref="C314:D314"/>
+    <mergeCell ref="C315:D315"/>
+    <mergeCell ref="C316:D316"/>
+    <mergeCell ref="C317:D317"/>
+    <mergeCell ref="C318:D318"/>
+    <mergeCell ref="C319:D319"/>
     <mergeCell ref="A6:F6"/>
     <mergeCell ref="H6:K6"/>
     <mergeCell ref="A1:K1"/>
@@ -16612,13 +16616,6 @@
     <mergeCell ref="A3:K3"/>
     <mergeCell ref="A4:K4"/>
     <mergeCell ref="J5:K5"/>
-    <mergeCell ref="C320:D320"/>
-    <mergeCell ref="C314:D314"/>
-    <mergeCell ref="C315:D315"/>
-    <mergeCell ref="C316:D316"/>
-    <mergeCell ref="C317:D317"/>
-    <mergeCell ref="C318:D318"/>
-    <mergeCell ref="C319:D319"/>
   </mergeCells>
   <phoneticPr fontId="84" type="noConversion"/>
   <printOptions horizontalCentered="1"/>

</xml_diff>